<commit_message>
chore: sync current workspace changes
</commit_message>
<xml_diff>
--- a/docs/客户表格定义.xlsx
+++ b/docs/客户表格定义.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mickey/project/PA-ALG/llm_client_search/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F3C2375-C2E5-E145-85A6-64181286687A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{425F440F-290F-7A47-9E54-CBA3356D11BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3220" yWindow="740" windowWidth="29400" windowHeight="16620" xr2:uid="{70D754B3-637B-8940-B50A-61FCD85FE96E}"/>
+    <workbookView xWindow="2440" yWindow="740" windowWidth="29400" windowHeight="16620" xr2:uid="{70D754B3-637B-8940-B50A-61FCD85FE96E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="已接入字段" sheetId="1" r:id="rId1"/>
+    <sheet name="未接入字段" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">已接入字段!$A$1:$J$48</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="224">
   <si>
     <t>字段分类</t>
   </si>
@@ -123,470 +124,687 @@
     <t>carNumber</t>
   </si>
   <si>
+    <t>证件类型</t>
+  </si>
+  <si>
+    <t>客户证件信息</t>
+  </si>
+  <si>
+    <t>证件到期时间</t>
+  </si>
+  <si>
+    <t>客户号</t>
+  </si>
+  <si>
+    <t>客户分类标签</t>
+  </si>
+  <si>
+    <t>客户价值</t>
+  </si>
+  <si>
+    <t>Hive</t>
+  </si>
+  <si>
+    <t>客户温度</t>
+  </si>
+  <si>
+    <t>客群标签(客户分群)</t>
+  </si>
+  <si>
+    <t>寿险VIP</t>
+  </si>
+  <si>
+    <t>存量客户类型</t>
+  </si>
+  <si>
+    <t>保单托管</t>
+  </si>
+  <si>
+    <t>持有产品类型</t>
+  </si>
+  <si>
+    <t>客户库主表, 险种基表, 险种表</t>
+  </si>
+  <si>
+    <t>待明确</t>
+  </si>
+  <si>
+    <t>客户库主表, 险种基表</t>
+  </si>
+  <si>
+    <t>查询app_client_buy_produc_Y</t>
+  </si>
+  <si>
+    <t>养老险产品</t>
+  </si>
+  <si>
+    <t>关联方</t>
+  </si>
+  <si>
+    <t>健康险</t>
+  </si>
+  <si>
+    <t>长险保单事件</t>
+  </si>
+  <si>
+    <t>年缴保费</t>
+  </si>
+  <si>
+    <t>范围匹配</t>
+  </si>
+  <si>
+    <t>短险保单事件</t>
+  </si>
+  <si>
+    <t>保单到期时间</t>
+  </si>
+  <si>
+    <t>会员等级</t>
+  </si>
+  <si>
+    <t>康养达标客户等级</t>
+  </si>
+  <si>
+    <t>客户家庭成员</t>
+  </si>
+  <si>
+    <t>成员关系</t>
+  </si>
+  <si>
+    <t>客户库-家庭关系表</t>
+  </si>
+  <si>
+    <t>成员性别</t>
+  </si>
+  <si>
+    <t>成员出生日期</t>
+  </si>
+  <si>
+    <t>保单信息</t>
+  </si>
+  <si>
+    <t>保单号</t>
+  </si>
+  <si>
+    <t>客户库-寿险保单关系表</t>
+  </si>
+  <si>
+    <t>产品总保额</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>insnoSumInsSeq</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>缴费期满</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>持有综拓产品类别</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>是否综拓理赔</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>occurPassPayRegst</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>validSinsMatuDate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>有效短险保单</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>validSinsPol</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>居家达标客户等级</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>臻享家医权益等级</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>格式: yyyy-MM-dd HH:mm:ss</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>男、女</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>博士后、大学专科、小学、博士研究生、中专、小学以下、大学本科生、初中、硕士研究生、高中</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>一般学生、武术指导、程序员、老师、医生</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>出生证、身份证、户口本、港澳台居住证、军人证、港澳台证、护照、外国人居留证</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>A1、A2、 A3、A4、B、C、D、E、F</t>
+  </si>
+  <si>
+    <t>高温、中温、低温、冷却</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gProductCode</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>hProductCode</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>奋斗青年、都市白领、新晋父母、社会中坚、邻退天命、慈爱祖辈、创业新贵、创富一代、荣耀高堂、承富二代、已退小康</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>原黄金VIP、原铂金VIP、黄金V1、黄金V2、黄金V3、铂金V1、铂金V2、钻石VIP、金钻VIP、黑钻VIP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>生财宝、智能星、金利多、平安永福、平安康泰、盛世金越</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>分红型、普通型、投资连结型、万能型、其他</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>定期寿险、护理保险、疾病保险、两全保险、年金保险、医疗保险、意外伤害保险、终身寿险</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>车险、非车险</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>一年期综合意外保险、一年期交通意外保险</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>e生保、安康、平安宝贝、i康保、i药保、海外、抗癌、尊享、尊优、舒享、其他</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>车辆交强险、车辆商业险、e生保、中高端医疗、合家欢、家财险、学平险、财富、健康、生活</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>是、否</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>综拓、O2O、意健险</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>居家潜客、v0.5、v1、v1.5、v2、v2.5、v3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>康养预达标会员、逸享会员、逸享PLUS会员、颐享家会员、臻享会员V1、臻享会员V2、臻享会员V3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>国内版、国际版</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>预达标、已达标</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>配偶、父母、子女、兄弟姐妹、法定、（外）祖父母、（外）孙子女</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>离婚、未婚、丧偶、已婚、未知</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>格式：数值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>产险产品</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>trusteeshipFlag</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>保单周年日</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>出生年月日</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>clientBirthday</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>familyRelation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>clientMobile</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>车辆型号</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>证件号</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>idNo</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>familyClientName</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>idValidDate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>effAppEndDate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>effAnniversaryDate</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>familyClientBirthday</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>寿险产品</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>marriSts</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>education</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>profName</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>assetsCondition</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>idType</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>newValueLabel</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>clientTemperature</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>clientGroupLabel</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>vipType</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>orphanType</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>productCode</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>pType</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>isBuyPregnancyCar</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>agentPerspProductType</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>familyClientSex</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>clientAge</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年龄</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>成员年龄</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>familyClientAge</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>birthdayMd</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在职有效客户、纯存续单客户、非纯存续单客户</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>持有产品类型</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>policyNo</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>clientNo</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>综拓理赔报案、综拓理赔结束</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>年收入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>annual_income</t>
+  </si>
+  <si>
+    <t>家庭收入</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>household_income</t>
+  </si>
+  <si>
+    <t>房产情况</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>real_estate_status</t>
+  </si>
+  <si>
+    <t>资产规模</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>asset_scale</t>
+  </si>
+  <si>
+    <t>产品名称</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>policies_product_name</t>
+  </si>
+  <si>
+    <t>保单生效日</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>policies_effective_date</t>
+  </si>
+  <si>
+    <t>保单状态</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>policies_status</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>投保日期</t>
+  </si>
+  <si>
+    <t>policies_insure_date</t>
+  </si>
+  <si>
+    <t>承保日期</t>
+  </si>
+  <si>
+    <t>policies_undwrt_date</t>
+  </si>
+  <si>
+    <t>应缴日</t>
+  </si>
+  <si>
+    <t>policies_pay_date</t>
+  </si>
+  <si>
+    <t>犹豫期时间</t>
+  </si>
+  <si>
+    <t>policies_cooling_off</t>
+  </si>
+  <si>
+    <t>policies_plan_fullname</t>
+  </si>
+  <si>
+    <t>policies_plan_abbr_name</t>
+  </si>
+  <si>
+    <t>policies_plan_type</t>
+  </si>
+  <si>
+    <t>投保人姓名</t>
+  </si>
+  <si>
+    <t>投保人手机号</t>
+  </si>
+  <si>
+    <t>被保人姓名</t>
+  </si>
+  <si>
+    <t>被保人手机号</t>
+  </si>
+  <si>
+    <t>受益人姓名</t>
+  </si>
+  <si>
+    <t>受益人手机号</t>
+  </si>
+  <si>
+    <t>生存金总金额</t>
+  </si>
+  <si>
+    <t>生存金已领取金额</t>
+  </si>
+  <si>
+    <t>生存金未领取金额</t>
+  </si>
+  <si>
+    <t>生存金已转入万能账户金额</t>
+  </si>
+  <si>
+    <t>生存金利息未领取总额</t>
+  </si>
+  <si>
+    <t>policies_applicant_name</t>
+  </si>
+  <si>
+    <t>policies_applicant_mobile</t>
+  </si>
+  <si>
+    <t>policies_insured_name</t>
+  </si>
+  <si>
+    <t>policies_insured_mobile</t>
+  </si>
+  <si>
+    <t>policies_beneficiary_name</t>
+  </si>
+  <si>
+    <t>policies_beneficiary_mobile</t>
+  </si>
+  <si>
+    <t>policies_survival_total_amount</t>
+  </si>
+  <si>
+    <t>policies_survival_claimed_amount</t>
+  </si>
+  <si>
+    <t>policies_survival_unclaimed_amount</t>
+  </si>
+  <si>
+    <t>policies_universal_acct_transfer</t>
+  </si>
+  <si>
+    <t>policies_survival_interest_total</t>
+  </si>
+  <si>
+    <t>投保险种简称</t>
+  </si>
+  <si>
+    <t>投保险种名称</t>
+  </si>
+  <si>
+    <t>投保险种类型</t>
+  </si>
+  <si>
+    <t>理赔时间</t>
+  </si>
+  <si>
+    <t>理赔案件号</t>
+  </si>
+  <si>
+    <t>理赔险种</t>
+  </si>
+  <si>
+    <t>理赔金额</t>
+  </si>
+  <si>
+    <t>格式：以P开头+15位数值的字符串，例如：P310000004303642</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>数值</t>
+  </si>
+  <si>
+    <t>有房、没房</t>
+  </si>
+  <si>
+    <t>取消、死亡理赔、展期、缴费有效、停效、到期终止、犹豫期退保、交清、减额交情、退保、转换终止、失效、终止效率、免交、迁出、人为停效、效力终止、预收、拒保、贷款超停、死亡有效、贷款超失、自垫有效、自垫停效、自垫失效、自垫交清、等待续保</t>
+  </si>
+  <si>
+    <t>持有产品类别</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>平安e生保医疗保险</t>
+  </si>
+  <si>
+    <t>e生保、安康、平安宝贝、i康保、i药保、海外、抗癌、尊享、尊优、舒享、其他</t>
+  </si>
+  <si>
+    <t>格式: yyyy-MM-dd HH:mm:ss</t>
+  </si>
+  <si>
+    <t>policies_claim_records_time</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>policies_claim_records_case_id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>policies_claim_records_amount</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>policies_claim_records_coverage</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>是否有车</t>
-  </si>
-  <si>
-    <t>证件类型</t>
-  </si>
-  <si>
-    <t>客户证件信息</t>
-  </si>
-  <si>
-    <t>证件到期时间</t>
-  </si>
-  <si>
-    <t>客户号</t>
-  </si>
-  <si>
-    <t>客户分类标签</t>
-  </si>
-  <si>
-    <t>客户价值</t>
-  </si>
-  <si>
-    <t>Hive</t>
-  </si>
-  <si>
-    <t>客户温度</t>
-  </si>
-  <si>
-    <t>客群标签(客户分群)</t>
-  </si>
-  <si>
-    <t>寿险VIP</t>
-  </si>
-  <si>
-    <t>存量客户类型</t>
-  </si>
-  <si>
-    <t>保单托管</t>
-  </si>
-  <si>
-    <t>持有产品类型</t>
-  </si>
-  <si>
-    <t>客户库主表, 险种基表, 险种表</t>
-  </si>
-  <si>
-    <t>待明确</t>
-  </si>
-  <si>
-    <t>客户库主表, 险种基表</t>
-  </si>
-  <si>
-    <t>查询app_client_buy_produc_Y</t>
-  </si>
-  <si>
-    <t>养老险产品</t>
-  </si>
-  <si>
-    <t>关联方</t>
-  </si>
-  <si>
-    <t>健康险</t>
-  </si>
-  <si>
-    <t>长险保单事件</t>
-  </si>
-  <si>
-    <t>年缴保费</t>
-  </si>
-  <si>
-    <t>范围匹配</t>
-  </si>
-  <si>
-    <t>短险保单事件</t>
-  </si>
-  <si>
-    <t>保单到期时间</t>
-  </si>
-  <si>
-    <t>会员等级</t>
-  </si>
-  <si>
-    <t>康养达标客户等级</t>
-  </si>
-  <si>
-    <t>客户家庭成员</t>
-  </si>
-  <si>
-    <t>成员关系</t>
-  </si>
-  <si>
-    <t>客户库-家庭关系表</t>
-  </si>
-  <si>
-    <t>成员性别</t>
-  </si>
-  <si>
-    <t>成员出生日期</t>
-  </si>
-  <si>
-    <t>保单信息</t>
-  </si>
-  <si>
-    <t>保单号</t>
-  </si>
-  <si>
-    <t>客户库-寿险保单关系表</t>
-  </si>
-  <si>
-    <t>amPremSeg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>产品总保额</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>insnoSumInsSeq</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>缴费期满</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>持有综拓产品类别</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>是否综拓理赔</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>occurPassPayRegst</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>validSinsMatuDate</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>有效短险保单</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>validSinsPol</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>居家达标客户等级</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>安有护权益等级</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>zhenxiangRunEquityGrade</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>zxjyEquityGrade</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>臻享家医权益等级</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>格式: yyyy-MM-dd HH:mm:ss</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>男、女</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>博士后、大学专科、小学、博士研究生、中专、小学以下、大学本科生、初中、硕士研究生、高中</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>一般学生、武术指导、程序员、老师、医生</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>出生证、身份证、户口本、港澳台居住证、军人证、港澳台证、护照、外国人居留证</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>A1、A2、 A3、A4、B、C、D、E、F</t>
-  </si>
-  <si>
-    <t>高温、中温、低温、冷却</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>gProductCode</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>hProductCode</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>奋斗青年、都市白领、新晋父母、社会中坚、邻退天命、慈爱祖辈、创业新贵、创富一代、荣耀高堂、承富二代、已退小康</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>原黄金VIP、原铂金VIP、黄金V1、黄金V2、黄金V3、铂金V1、铂金V2、钻石VIP、金钻VIP、黑钻VIP</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>生财宝、智能星、金利多、平安永福、平安康泰、盛世金越</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>分红型、普通型、投资连结型、万能型、其他</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>定期寿险、护理保险、疾病保险、两全保险、年金保险、医疗保险、意外伤害保险、终身寿险</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>车险、非车险</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>一年期综合意外保险、一年期交通意外保险</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>e生保、安康、平安宝贝、i康保、i药保、海外、抗癌、尊享、尊优、舒享、其他</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>车辆交强险、车辆商业险、e生保、中高端医疗、合家欢、家财险、学平险、财富、健康、生活</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>是、否</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>综拓、O2O、意健险</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>居家潜客、v0.5、v1、v1.5、v2、v2.5、v3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>康养预达标会员、逸享会员、逸享PLUS会员、颐享家会员、臻享会员V1、臻享会员V2、臻享会员V3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>国内版、国际版</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>预达标、已达标</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>配偶、父母、子女、兄弟姐妹、法定、（外）祖父母、（外）孙子女</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>离婚、未婚、丧偶、已婚、未知</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>有车、没车</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>格式：数值</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>产险产品</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>trusteeshipFlag</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>保单周年日</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>出生年月日</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>clientBirthday</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>familyRelation</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>clientMobile</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>车辆型号</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>证件号</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>idNo</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>familyClientName</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>idValidDate</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>effAppEndDate</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>effAnniversaryDate</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>familyClientBirthday</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>寿险产品</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>marriSts</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>education</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>profName</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>assetsCondition</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>idType</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>newValueLabel</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>clientTemperature</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>clientGroupLabel</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>vipType</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>orphanType</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>productCode</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>pType</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>pcCategory</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>isBuyPregnancyCar</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>agentPerspProductType</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>jujiaClientGrade</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>kangyangClientGrade</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>familyClientSex</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>clientAge</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>姓名</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>年龄</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>成员年龄</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>familyClientAge</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>birthdayMd</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>在职有效客户、纯存续单客户、非纯存续单客户</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>持有产品品类</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>持有产品类型</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>clientName</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>policyNo</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>clientNo</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>综拓理赔报案、综拓理赔结束</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>annPremSeg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>pCategory</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>安有护权益</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>有房、有车、有房有车、无房无车</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>searchZxjyEquityGrade</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>searchZhenxiangRunEquityGrade</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>searchKangyangClientGrade</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>searchJujiaClientGrade</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>searchClientName</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>成员姓名</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>成员手机号</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>familyClientMobile</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -594,7 +812,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -618,8 +836,34 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Google Sans"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="等线"/>
+      <family val="4"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Google Sans"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="4"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -630,6 +874,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFD"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -647,7 +903,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -655,6 +911,39 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -971,7 +1260,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B00495F1-53EB-9F44-BBB4-156CB62E6D7B}">
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="13.6640625" customWidth="1"/>
@@ -1020,7 +1309,7 @@
         <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>153</v>
+        <v>220</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
@@ -1049,7 +1338,7 @@
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
@@ -1090,7 +1379,7 @@
         <v>13</v>
       </c>
       <c r="H4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="I4" t="s">
         <v>19</v>
@@ -1104,10 +1393,10 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C5" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="D5" t="s">
         <v>12</v>
@@ -1122,7 +1411,7 @@
         <v>13</v>
       </c>
       <c r="H5" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="I5" t="s">
         <v>19</v>
@@ -1139,7 +1428,7 @@
         <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="D6" t="s">
         <v>21</v>
@@ -1168,10 +1457,10 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="C7" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="E7" t="s">
         <v>23</v>
@@ -1194,7 +1483,7 @@
         <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="D8" t="s">
         <v>12</v>
@@ -1209,7 +1498,7 @@
         <v>13</v>
       </c>
       <c r="H8" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="J8" t="s">
         <v>15</v>
@@ -1223,7 +1512,7 @@
         <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
@@ -1238,7 +1527,7 @@
         <v>13</v>
       </c>
       <c r="H9" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="I9" t="s">
         <v>19</v>
@@ -1255,7 +1544,7 @@
         <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1270,7 +1559,7 @@
         <v>13</v>
       </c>
       <c r="H10" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="I10" t="s">
         <v>19</v>
@@ -1279,61 +1568,61 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
-      <c r="A11" t="s">
+    <row r="11" spans="1:10" s="1" customFormat="1">
+      <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
-        <v>117</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="B11" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" t="s">
-        <v>13</v>
-      </c>
-      <c r="I11" t="s">
+      <c r="E11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
-      <c r="A12" t="s">
+    <row r="12" spans="1:10" s="1" customFormat="1">
+      <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E12" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I12" t="s">
+      <c r="E12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="1" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1342,10 +1631,10 @@
         <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>211</v>
       </c>
       <c r="C13" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
@@ -1360,7 +1649,7 @@
         <v>13</v>
       </c>
       <c r="H13" t="s">
-        <v>108</v>
+        <v>215</v>
       </c>
       <c r="J13" t="s">
         <v>15</v>
@@ -1371,10 +1660,10 @@
         <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C14" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
@@ -1389,7 +1678,7 @@
         <v>13</v>
       </c>
       <c r="H14" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="I14" t="s">
         <v>19</v>
@@ -1400,13 +1689,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B15" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="C15" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
@@ -1429,13 +1718,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" t="s">
         <v>33</v>
       </c>
-      <c r="B16" t="s">
-        <v>34</v>
-      </c>
       <c r="C16" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
@@ -1450,7 +1739,7 @@
         <v>13</v>
       </c>
       <c r="H16" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="I16" t="s">
         <v>19</v>
@@ -1464,10 +1753,10 @@
         <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C17" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
@@ -1490,17 +1779,17 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" t="s">
         <v>36</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
+        <v>125</v>
+      </c>
+      <c r="D18" t="s">
         <v>37</v>
       </c>
-      <c r="C18" t="s">
-        <v>131</v>
-      </c>
-      <c r="D18" t="s">
-        <v>38</v>
-      </c>
       <c r="E18" t="s">
         <v>13</v>
       </c>
@@ -1511,7 +1800,7 @@
         <v>13</v>
       </c>
       <c r="H18" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="I18" t="s">
         <v>19</v>
@@ -1522,16 +1811,16 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C19" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E19" t="s">
         <v>13</v>
@@ -1543,7 +1832,7 @@
         <v>13</v>
       </c>
       <c r="H19" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="I19" t="s">
         <v>19</v>
@@ -1554,16 +1843,16 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B20" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C20" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E20" t="s">
         <v>13</v>
@@ -1575,7 +1864,7 @@
         <v>13</v>
       </c>
       <c r="H20" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="I20" t="s">
         <v>19</v>
@@ -1586,13 +1875,13 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C21" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="D21" t="s">
         <v>12</v>
@@ -1607,7 +1896,7 @@
         <v>13</v>
       </c>
       <c r="H21" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="I21" t="s">
         <v>19</v>
@@ -1618,16 +1907,16 @@
     </row>
     <row r="22" spans="1:10">
       <c r="A22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B22" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C22" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E22" t="s">
         <v>13</v>
@@ -1639,7 +1928,7 @@
         <v>13</v>
       </c>
       <c r="H22" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="I22" t="s">
         <v>19</v>
@@ -1650,16 +1939,16 @@
     </row>
     <row r="23" spans="1:10">
       <c r="A23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C23" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E23" t="s">
         <v>13</v>
@@ -1671,7 +1960,7 @@
         <v>13</v>
       </c>
       <c r="H23" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="I23" t="s">
         <v>19</v>
@@ -1682,48 +1971,48 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" t="s">
+        <v>119</v>
+      </c>
+      <c r="C24" t="s">
+        <v>130</v>
+      </c>
+      <c r="D24" t="s">
         <v>44</v>
       </c>
-      <c r="B24" t="s">
-        <v>125</v>
-      </c>
-      <c r="C24" t="s">
-        <v>136</v>
-      </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F24" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" t="s">
+        <v>13</v>
+      </c>
+      <c r="H24" t="s">
+        <v>88</v>
+      </c>
+      <c r="I24" t="s">
         <v>45</v>
       </c>
-      <c r="E24" t="s">
-        <v>23</v>
-      </c>
-      <c r="F24" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" t="s">
-        <v>13</v>
-      </c>
-      <c r="H24" t="s">
-        <v>93</v>
-      </c>
-      <c r="I24" t="s">
-        <v>46</v>
-      </c>
       <c r="J24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B25" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="C25" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="D25" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E25" t="s">
         <v>23</v>
@@ -1735,187 +2024,187 @@
         <v>13</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="I25" t="s">
+        <v>45</v>
+      </c>
+      <c r="J25" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" s="13" customFormat="1">
+      <c r="A26" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="D26" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="J25" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10">
-      <c r="A26" t="s">
-        <v>44</v>
-      </c>
-      <c r="B26" t="s">
-        <v>151</v>
-      </c>
-      <c r="C26" t="s">
-        <v>138</v>
-      </c>
-      <c r="D26" t="s">
-        <v>47</v>
-      </c>
-      <c r="E26" t="s">
-        <v>23</v>
-      </c>
-      <c r="F26" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" t="s">
-        <v>13</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="I26" t="s">
-        <v>46</v>
-      </c>
-      <c r="J26" t="s">
-        <v>46</v>
+      <c r="E26" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="I26" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="J26" s="13" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B27" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="C27" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D27" t="s">
+        <v>47</v>
+      </c>
+      <c r="E27" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" t="s">
+        <v>13</v>
+      </c>
+      <c r="H27" t="s">
+        <v>91</v>
+      </c>
+      <c r="I27" t="s">
+        <v>45</v>
+      </c>
+      <c r="J27" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" s="1" customFormat="1">
+      <c r="A28" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E27" t="s">
-        <v>13</v>
-      </c>
-      <c r="F27" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" t="s">
-        <v>13</v>
-      </c>
-      <c r="H27" t="s">
-        <v>96</v>
-      </c>
-      <c r="I27" t="s">
-        <v>46</v>
-      </c>
-      <c r="J27" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10">
-      <c r="A28" t="s">
-        <v>44</v>
-      </c>
-      <c r="B28" t="s">
+      <c r="C28" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C28" t="s">
-        <v>89</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="E28" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" s="1" customFormat="1" ht="15" customHeight="1">
+      <c r="A29" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E28" t="s">
-        <v>13</v>
-      </c>
-      <c r="F28" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" t="s">
-        <v>13</v>
-      </c>
-      <c r="H28" t="s">
-        <v>97</v>
-      </c>
-      <c r="I28" t="s">
-        <v>46</v>
-      </c>
-      <c r="J28" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="15" customHeight="1">
-      <c r="A29" t="s">
-        <v>44</v>
-      </c>
-      <c r="B29" t="s">
+      <c r="C29" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" s="13" customFormat="1">
+      <c r="A30" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="C29" t="s">
-        <v>90</v>
-      </c>
-      <c r="D29" t="s">
-        <v>50</v>
-      </c>
-      <c r="E29" t="s">
-        <v>13</v>
-      </c>
-      <c r="F29" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" t="s">
-        <v>13</v>
-      </c>
-      <c r="H29" t="s">
-        <v>98</v>
-      </c>
-      <c r="I29" t="s">
-        <v>46</v>
-      </c>
-      <c r="J29" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" s="1" customFormat="1">
-      <c r="A30" s="1" t="s">
+      <c r="B30" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="C30" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H30" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="I30" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="C30" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="I30" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="J30" s="1" t="s">
+      <c r="J30" s="13" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B31" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C31" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D31" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E31" t="s">
         <v>13</v>
@@ -1927,27 +2216,27 @@
         <v>13</v>
       </c>
       <c r="H31" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="I31" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J31" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B32" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C32" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="D32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E32" t="s">
         <v>13</v>
@@ -1959,7 +2248,7 @@
         <v>13</v>
       </c>
       <c r="H32" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="I32" t="s">
         <v>19</v>
@@ -1970,16 +2259,16 @@
     </row>
     <row r="33" spans="1:10">
       <c r="A33" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B33" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C33" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="D33" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E33" t="s">
         <v>13</v>
@@ -1991,7 +2280,7 @@
         <v>13</v>
       </c>
       <c r="H33" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="I33" t="s">
         <v>19</v>
@@ -2002,16 +2291,16 @@
     </row>
     <row r="34" spans="1:10">
       <c r="A34" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B34" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C34" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="D34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E34" t="s">
         <v>13</v>
@@ -2023,7 +2312,7 @@
         <v>13</v>
       </c>
       <c r="H34" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="I34" t="s">
         <v>19</v>
@@ -2034,16 +2323,16 @@
     </row>
     <row r="35" spans="1:10">
       <c r="A35" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C35" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D35" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E35" t="s">
         <v>13</v>
@@ -2055,7 +2344,7 @@
         <v>13</v>
       </c>
       <c r="H35" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="I35" t="s">
         <v>19</v>
@@ -2064,50 +2353,50 @@
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:10" s="2" customFormat="1">
-      <c r="A36" s="2" t="s">
+    <row r="36" spans="1:10" s="12" customFormat="1">
+      <c r="A36" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B36" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="I36" s="2" t="s">
+      <c r="C36" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="G36" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H36" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="I36" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="J36" s="2" t="s">
+      <c r="J36" s="12" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B37" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C37" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D37" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E37" t="s">
         <v>13</v>
@@ -2119,7 +2408,7 @@
         <v>13</v>
       </c>
       <c r="H37" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="I37" t="s">
         <v>19</v>
@@ -2130,16 +2419,16 @@
     </row>
     <row r="38" spans="1:10">
       <c r="A38" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B38" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C38" t="s">
-        <v>141</v>
+        <v>219</v>
       </c>
       <c r="D38" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E38" t="s">
         <v>13</v>
@@ -2151,7 +2440,7 @@
         <v>13</v>
       </c>
       <c r="H38" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="I38" t="s">
         <v>19</v>
@@ -2162,16 +2451,16 @@
     </row>
     <row r="39" spans="1:10">
       <c r="A39" t="s">
+        <v>56</v>
+      </c>
+      <c r="B39" t="s">
         <v>57</v>
       </c>
-      <c r="B39" t="s">
-        <v>58</v>
-      </c>
       <c r="C39" t="s">
-        <v>142</v>
+        <v>218</v>
       </c>
       <c r="D39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E39" t="s">
         <v>13</v>
@@ -2183,7 +2472,7 @@
         <v>13</v>
       </c>
       <c r="H39" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="I39" t="s">
         <v>19</v>
@@ -2194,16 +2483,16 @@
     </row>
     <row r="40" spans="1:10">
       <c r="A40" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B40" t="s">
-        <v>78</v>
+        <v>214</v>
       </c>
       <c r="C40" t="s">
-        <v>79</v>
+        <v>217</v>
       </c>
       <c r="D40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E40" t="s">
         <v>13</v>
@@ -2215,7 +2504,7 @@
         <v>13</v>
       </c>
       <c r="H40" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="I40" t="s">
         <v>19</v>
@@ -2226,16 +2515,16 @@
     </row>
     <row r="41" spans="1:10">
       <c r="A41" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B41" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C41" t="s">
-        <v>80</v>
+        <v>216</v>
       </c>
       <c r="D41" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E41" t="s">
         <v>13</v>
@@ -2247,7 +2536,7 @@
         <v>13</v>
       </c>
       <c r="H41" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="I41" t="s">
         <v>19</v>
@@ -2258,17 +2547,17 @@
     </row>
     <row r="42" spans="1:10">
       <c r="A42" t="s">
+        <v>58</v>
+      </c>
+      <c r="B42" t="s">
         <v>59</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
+        <v>109</v>
+      </c>
+      <c r="D42" t="s">
         <v>60</v>
       </c>
-      <c r="C42" t="s">
-        <v>115</v>
-      </c>
-      <c r="D42" t="s">
-        <v>61</v>
-      </c>
       <c r="E42" t="s">
         <v>13</v>
       </c>
@@ -2279,7 +2568,7 @@
         <v>13</v>
       </c>
       <c r="H42" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="I42" t="s">
         <v>19</v>
@@ -2290,16 +2579,16 @@
     </row>
     <row r="43" spans="1:10">
       <c r="A43" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B43" t="s">
-        <v>145</v>
+        <v>221</v>
       </c>
       <c r="C43" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D43" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E43" t="s">
         <v>23</v>
@@ -2319,16 +2608,16 @@
     </row>
     <row r="44" spans="1:10">
       <c r="A44" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B44" t="s">
-        <v>62</v>
+        <v>222</v>
       </c>
       <c r="C44" t="s">
-        <v>143</v>
+        <v>223</v>
       </c>
       <c r="D44" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E44" t="s">
         <v>13</v>
@@ -2338,9 +2627,6 @@
       </c>
       <c r="G44" t="s">
         <v>13</v>
-      </c>
-      <c r="H44" t="s">
-        <v>83</v>
       </c>
       <c r="I44" t="s">
         <v>19</v>
@@ -2351,85 +2637,120 @@
     </row>
     <row r="45" spans="1:10">
       <c r="A45" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B45" t="s">
-        <v>147</v>
+        <v>61</v>
       </c>
       <c r="C45" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="D45" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E45" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F45" t="s">
         <v>13</v>
       </c>
       <c r="G45" t="s">
         <v>13</v>
+      </c>
+      <c r="H45" t="s">
+        <v>78</v>
+      </c>
+      <c r="I45" t="s">
+        <v>19</v>
+      </c>
+      <c r="J45" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="46" spans="1:10">
       <c r="A46" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B46" t="s">
-        <v>63</v>
+        <v>137</v>
       </c>
       <c r="C46" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="D46" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E46" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F46" t="s">
         <v>13</v>
       </c>
       <c r="G46" t="s">
         <v>13</v>
-      </c>
-      <c r="H46" t="s">
-        <v>82</v>
-      </c>
-      <c r="I46" t="s">
-        <v>19</v>
-      </c>
-      <c r="J46" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="47" spans="1:10">
       <c r="A47" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="B47" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C47" t="s">
-        <v>154</v>
+        <v>118</v>
       </c>
       <c r="D47" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E47" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F47" t="s">
         <v>13</v>
       </c>
       <c r="G47" t="s">
         <v>13</v>
+      </c>
+      <c r="H47" t="s">
+        <v>77</v>
       </c>
       <c r="I47" t="s">
         <v>19</v>
       </c>
       <c r="J47" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10">
+      <c r="A48" t="s">
+        <v>63</v>
+      </c>
+      <c r="B48" t="s">
+        <v>64</v>
+      </c>
+      <c r="C48" t="s">
+        <v>142</v>
+      </c>
+      <c r="D48" t="s">
+        <v>65</v>
+      </c>
+      <c r="E48" t="s">
+        <v>23</v>
+      </c>
+      <c r="F48" t="s">
+        <v>13</v>
+      </c>
+      <c r="G48" t="s">
+        <v>13</v>
+      </c>
+      <c r="H48" t="s">
+        <v>199</v>
+      </c>
+      <c r="I48" t="s">
+        <v>19</v>
+      </c>
+      <c r="J48" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2438,4 +2759,780 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE826B49-0248-F348-BAF6-825D34FC36A5}">
+  <dimension ref="A1:J30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="4" max="4" width="51.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+    </row>
+    <row r="5" spans="1:10" s="1" customFormat="1">
+      <c r="A5" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+    </row>
+    <row r="6" spans="1:10" s="1" customFormat="1">
+      <c r="A6" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="I9" s="4"/>
+      <c r="J9" s="4"/>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
+    </row>
+    <row r="16" spans="1:10" ht="30">
+      <c r="A16" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+    </row>
+    <row r="17" spans="1:10">
+      <c r="A17" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="A18" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+    </row>
+    <row r="20" spans="1:10">
+      <c r="A20" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+    </row>
+    <row r="21" spans="1:10">
+      <c r="A21" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+    </row>
+    <row r="22" spans="1:10">
+      <c r="A22" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D22" s="3"/>
+      <c r="E22" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+    </row>
+    <row r="23" spans="1:10">
+      <c r="A23" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="D23" s="3"/>
+      <c r="E23" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+    </row>
+    <row r="24" spans="1:10">
+      <c r="A24" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D24" s="3"/>
+      <c r="E24" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+    </row>
+    <row r="25" spans="1:10">
+      <c r="A25" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D25" s="3"/>
+      <c r="E25" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="D26" s="3"/>
+      <c r="E26" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+    </row>
+    <row r="28" spans="1:10">
+      <c r="A28" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="D28" s="3"/>
+      <c r="E28" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+    </row>
+    <row r="29" spans="1:10">
+      <c r="A29" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="D29" s="3"/>
+      <c r="E29" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+    </row>
+    <row r="30" spans="1:10">
+      <c r="A30" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="D30" s="3"/>
+      <c r="E30" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H30" s="4"/>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>